<commit_message>
Add monthly owner statement PDF generator
- New generate_owner_statements.py script using reportlab
- Produces per-owner PDFs with trips, payments, and net due
- CLI supports --month, --owner, --list-months, and --output
- Add Statements sheet to workbook with usage instructions
- Add requirements.txt and gitignore generated PDF output

Co-authored-by: Shyam <shyam.nexus@gmail.com>
</commit_message>
<xml_diff>
--- a/HARIOM LOGISTICS - Automated.xlsx
+++ b/HARIOM LOGISTICS - Automated.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Owner Ledger" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Freight Bills" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Payments" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Pump Account" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Master Data" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Statements" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Pump Account" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Master Data" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="DD-MMM-YYYY"/>
     <numFmt numFmtId="166" formatCode="DD-MMM-YYYY HH:MM"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,6 +65,14 @@
     <font>
       <color rgb="00444444"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -110,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,6 +135,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -598,7 +609,7 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>46201.5166009442</v>
+        <v>46201.51878355152</v>
       </c>
     </row>
     <row r="19">
@@ -26771,6 +26782,171 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>HARIOM LOGISTICS — OWNER STATEMENT PDFs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Generate monthly PDF statements per truck owner from Trip Log and Payments data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>COMMAND</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>python3 generate_owner_statements.py --month 2026-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Command</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>List available months</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>python3 generate_owner_statements.py --list-months</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Generate all owners (June 2026)</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>python3 generate_owner_statements.py --month 2026-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Generate one owner only</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>python3 generate_owner_statements.py --month 2026-06 --owner VINEET</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Custom output folder</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>python3 generate_owner_statements.py --month 2026-06 --output ./statements</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>OUTPUT LOCATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PDFs are saved to: statements/YYYY-MM/YYYY-MM_OwnerName_statement.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>EACH PDF INCLUDES</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• Trip details: LR, date, party, destination, truck, freight, commission, balance, PAHUNCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• Trip summary: totals for freight, commission, munsiyana, balance payable</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>• Payments received that month</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>• Account summary: balance payable − payments = net due</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -27752,7 +27928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27816,32 +27992,32 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>PARTIES (Sold To)</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>DESTINATIONS</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>TRUCKS</t>
         </is>
       </c>
-      <c r="J3" s="13" t="inlineStr">
+      <c r="J3" s="15" t="inlineStr">
         <is>
           <t>OWNERS</t>
         </is>
       </c>
-      <c r="L3" s="13" t="inlineStr">
+      <c r="L3" s="15" t="inlineStr">
         <is>
           <t>STATUS LISTS</t>
         </is>
       </c>
-      <c r="P3" s="13" t="inlineStr">
+      <c r="P3" s="15" t="inlineStr">
         <is>
           <t>TRIP BILL REFS</t>
         </is>

</xml_diff>

<commit_message>
Fix conditional formatting colors in Excel workbook
- Replace date-based rules with ISBLANK checks that work reliably
- Add red/yellow row highlights and zebra striping on Trip Log
- Add color rules on Owner Ledger (net due) and Freight Bills (EPOD/pending)
- Set explicit fill colors with fgColor and bgColor for Excel compatibility

Co-authored-by: Shyam <shyam.nexus@gmail.com>
</commit_message>
<xml_diff>
--- a/HARIOM LOGISTICS - Automated.xlsx
+++ b/HARIOM LOGISTICS - Automated.xlsx
@@ -151,18 +151,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFEB9C"/>
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
+          <fgColor rgb="00FFEB9C"/>
+          <bgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F2F7FB"/>
+          <bgColor rgb="00F2F7FB"/>
         </patternFill>
       </fill>
     </dxf>
@@ -618,7 +628,7 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>46201.52168413039</v>
+        <v>46201.62031331599</v>
       </c>
     </row>
     <row r="19">
@@ -659,7 +669,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>5. Yellow rows = PAHUNCH overdue. Red rows = Bill Ref missing on a trip with freight.</t>
+          <t>5. Row colors on Trip Log: Yellow = PAHUNCH missing. Red = Bill Ref missing.</t>
         </is>
       </c>
     </row>
@@ -717,7 +727,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Tip: Use dropdown arrows on Party, Destination &amp; Truck columns. Owner, Commission &amp; Balance auto-fill when you pick a truck. Requires Microsoft Excel.</t>
+          <t>Yellow = PAHUNCH missing. Red = Bill Ref missing. Pick Party, Destination &amp; Truck from dropdown arrows. Requires Microsoft Excel.</t>
         </is>
       </c>
     </row>
@@ -24485,11 +24495,14 @@
     <mergeCell ref="A2:T2"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:T503">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND($B4&lt;&gt;"", $P4="", $B4&lt;TODAY()-2)</formula>
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>AND($A4&lt;&gt;"",$G4&lt;&gt;"",ISBLANK($Q4))</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>AND($Q4="", $I4&lt;&gt;"")</formula>
+    <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="1">
+      <formula>AND($A4&lt;&gt;"",$G4&lt;&gt;"",ISBLANK($P4))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="0">
+      <formula>AND(MOD(ROW(),2)=0,$A4&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
@@ -24867,7 +24880,7 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:J9">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="0">
       <formula>$H5&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -24983,7 +24996,7 @@
           <t>HO/JUN/01</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>1 EPOD</t>
         </is>
@@ -25032,7 +25045,7 @@
           <t>HO/JUN/02</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>2 EPOD</t>
         </is>
@@ -25081,7 +25094,7 @@
           <t>HO/JUN/03</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -25130,7 +25143,7 @@
           <t>HO/JUN/04</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>4 EPOD</t>
         </is>
@@ -25179,7 +25192,7 @@
           <t>HO/JUN/05</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -25228,7 +25241,7 @@
           <t>HO/JUN/06</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -25277,7 +25290,7 @@
           <t>HO/JUN/07</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>7 EPOD</t>
         </is>
@@ -25326,7 +25339,7 @@
           <t>HO/JUN/08</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>8 EPOD</t>
         </is>
@@ -25375,7 +25388,7 @@
           <t>HO/JUN/09</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>9 EPOD</t>
         </is>
@@ -25424,7 +25437,7 @@
           <t>HO/JUN/10</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -25473,7 +25486,7 @@
           <t>HO/JUN/11</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>11</t>
         </is>
@@ -25514,6 +25527,7 @@
       </c>
     </row>
     <row r="16">
+      <c r="C16" s="9" t="n"/>
       <c r="D16" s="9">
         <f>IF(C16="","",SUMIF('Trip Log'!$Q$4:$Q$502,C16,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25538,6 +25552,7 @@
       </c>
     </row>
     <row r="17">
+      <c r="C17" s="9" t="n"/>
       <c r="D17" s="9">
         <f>IF(C17="","",SUMIF('Trip Log'!$Q$4:$Q$502,C17,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25562,6 +25577,7 @@
       </c>
     </row>
     <row r="18">
+      <c r="C18" s="9" t="n"/>
       <c r="D18" s="9">
         <f>IF(C18="","",SUMIF('Trip Log'!$Q$4:$Q$502,C18,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25586,6 +25602,7 @@
       </c>
     </row>
     <row r="19">
+      <c r="C19" s="9" t="n"/>
       <c r="D19" s="9">
         <f>IF(C19="","",SUMIF('Trip Log'!$Q$4:$Q$502,C19,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25610,6 +25627,7 @@
       </c>
     </row>
     <row r="20">
+      <c r="C20" s="9" t="n"/>
       <c r="D20" s="9">
         <f>IF(C20="","",SUMIF('Trip Log'!$Q$4:$Q$502,C20,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25634,6 +25652,7 @@
       </c>
     </row>
     <row r="21">
+      <c r="C21" s="9" t="n"/>
       <c r="D21" s="9">
         <f>IF(C21="","",SUMIF('Trip Log'!$Q$4:$Q$502,C21,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25658,6 +25677,7 @@
       </c>
     </row>
     <row r="22">
+      <c r="C22" s="9" t="n"/>
       <c r="D22" s="9">
         <f>IF(C22="","",SUMIF('Trip Log'!$Q$4:$Q$502,C22,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25682,6 +25702,7 @@
       </c>
     </row>
     <row r="23">
+      <c r="C23" s="9" t="n"/>
       <c r="D23" s="9">
         <f>IF(C23="","",SUMIF('Trip Log'!$Q$4:$Q$502,C23,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25706,6 +25727,7 @@
       </c>
     </row>
     <row r="24">
+      <c r="C24" s="9" t="n"/>
       <c r="D24" s="9">
         <f>IF(C24="","",SUMIF('Trip Log'!$Q$4:$Q$502,C24,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25730,6 +25752,7 @@
       </c>
     </row>
     <row r="25">
+      <c r="C25" s="9" t="n"/>
       <c r="D25" s="9">
         <f>IF(C25="","",SUMIF('Trip Log'!$Q$4:$Q$502,C25,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25754,6 +25777,7 @@
       </c>
     </row>
     <row r="26">
+      <c r="C26" s="9" t="n"/>
       <c r="D26" s="9">
         <f>IF(C26="","",SUMIF('Trip Log'!$Q$4:$Q$502,C26,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25778,6 +25802,7 @@
       </c>
     </row>
     <row r="27">
+      <c r="C27" s="9" t="n"/>
       <c r="D27" s="9">
         <f>IF(C27="","",SUMIF('Trip Log'!$Q$4:$Q$502,C27,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25802,6 +25827,7 @@
       </c>
     </row>
     <row r="28">
+      <c r="C28" s="9" t="n"/>
       <c r="D28" s="9">
         <f>IF(C28="","",SUMIF('Trip Log'!$Q$4:$Q$502,C28,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25826,6 +25852,7 @@
       </c>
     </row>
     <row r="29">
+      <c r="C29" s="9" t="n"/>
       <c r="D29" s="9">
         <f>IF(C29="","",SUMIF('Trip Log'!$Q$4:$Q$502,C29,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25850,6 +25877,7 @@
       </c>
     </row>
     <row r="30">
+      <c r="C30" s="9" t="n"/>
       <c r="D30" s="9">
         <f>IF(C30="","",SUMIF('Trip Log'!$Q$4:$Q$502,C30,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25874,6 +25902,7 @@
       </c>
     </row>
     <row r="31">
+      <c r="C31" s="9" t="n"/>
       <c r="D31" s="9">
         <f>IF(C31="","",SUMIF('Trip Log'!$Q$4:$Q$502,C31,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25898,6 +25927,7 @@
       </c>
     </row>
     <row r="32">
+      <c r="C32" s="9" t="n"/>
       <c r="D32" s="9">
         <f>IF(C32="","",SUMIF('Trip Log'!$Q$4:$Q$502,C32,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25922,6 +25952,7 @@
       </c>
     </row>
     <row r="33">
+      <c r="C33" s="9" t="n"/>
       <c r="D33" s="9">
         <f>IF(C33="","",SUMIF('Trip Log'!$Q$4:$Q$502,C33,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25946,6 +25977,7 @@
       </c>
     </row>
     <row r="34">
+      <c r="C34" s="9" t="n"/>
       <c r="D34" s="9">
         <f>IF(C34="","",SUMIF('Trip Log'!$Q$4:$Q$502,C34,'Trip Log'!$I$4:$I$502))</f>
         <v/>
@@ -25995,6 +26027,14 @@
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
   </mergeCells>
+  <conditionalFormatting sqref="A5:L34">
+    <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="0">
+      <formula>$G5="NO"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
+      <formula>$L5="PENDING"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="C5:C34" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." promptTitle="Dropdown" prompt="Click the arrow and select from the list" type="list">
       <formula1>=HL_BillRefs</formula1>

</xml_diff>